<commit_message>
Fixes to splitting problem with cvxlab
Introduce parameters to control the cvxlab optimization: only_input_data_gen and solver_parameter parameters added to Database.add_sectors, and updated call sites to either create cvxlab input files (without running the solver) or run the optimizer.
Implemented _create_input_data_for_cvxlab in mario/tools/cvxlab/models.py to populate cvxlab input sheets/CSVs from MARIO matrices and split metadata.
Extended _optimize_in_cvxlab to accept solver_parameter and pass MOSEK tolerance parameters when provided. Wire-up stores optimized matrices under 'split_cvxlab' and preserves necessary fallback matrices; also add history/log messages.
Minor excel handler updates: import of tolerance templates.
</commit_message>
<xml_diff>
--- a/mario/tools/cvxlab/Split_sectors/model_settings.xlsx
+++ b/mario/tools/cvxlab/Split_sectors/model_settings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/tools/cvxlab/Split_sectors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="97" documentId="8_{B691EA13-93EB-40C9-9646-E9A649F80B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{272BEC8D-C78C-47C1-AC96-88A254E65525}"/>
+  <xr:revisionPtr revIDLastSave="100" documentId="8_{B691EA13-93EB-40C9-9646-E9A649F80B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46476FA0-DCC0-4625-BF33-79EDBFC68A39}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10130" yWindow="-21710" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="problem" sheetId="5" r:id="rId1"/>
@@ -328,9 +328,6 @@
     <t>Znew0_use_st_pn</t>
   </si>
   <si>
-    <t>Znew_supply_imp&gt;=0</t>
-  </si>
-  <si>
     <t>Znew_use_st_pn&gt;=0</t>
   </si>
   <si>
@@ -541,9 +538,6 @@
     <t>Constraint 3-: column sum</t>
   </si>
   <si>
-    <t>tran(I_rs_from_to_n@Xnew_n) &gt;= (I_stable @ Znew_use_n+ I_pn @ Znew_supply_col + VA_n)*(1+delta)</t>
-  </si>
-  <si>
     <t>tran(I_rs_from_to_n@Xnew_n) &lt;= (I_stable @ Znew_use_n+ I_pn @ Znew_supply_col + VA_n)*(1+delta)</t>
   </si>
   <si>
@@ -557,6 +551,12 @@
   </si>
   <si>
     <t>Constraint 4+: trade balance</t>
+  </si>
+  <si>
+    <t>tran(I_rs_from_to_n@Xnew_n) &gt;= (I_stable @ Znew_use_n+ I_pn @ Znew_supply_col + VA_n)*(1-delta)</t>
+  </si>
+  <si>
+    <t>Znew_supply&gt;=0</t>
   </si>
 </sst>
 </file>
@@ -998,12 +998,12 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
-        <v>97</v>
+        <v>173</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>90</v>
@@ -1011,7 +1011,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>89</v>
@@ -1027,130 +1027,130 @@
     </row>
     <row r="6" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>148</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
+        <v>153</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C15" t="s">
+        <v>160</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>161</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C16" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C17" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C18" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C19" s="7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C20" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C21" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -1194,7 +1194,7 @@
         <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -1205,7 +1205,7 @@
         <v>18</v>
       </c>
       <c r="E3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -1226,7 +1226,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B6" t="s">
         <v>26</v>
@@ -1234,13 +1234,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E7" t="s">
         <v>140</v>
-      </c>
-      <c r="E7" t="s">
-        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -1303,10 +1303,10 @@
         <v>25</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
@@ -1328,10 +1328,10 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" t="s">
+        <v>118</v>
+      </c>
+      <c r="J2" t="s">
         <v>119</v>
-      </c>
-      <c r="J2" t="s">
-        <v>120</v>
       </c>
       <c r="K2" s="8" t="s">
         <v>36</v>
@@ -1468,13 +1468,13 @@
         <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F7" t="s">
         <v>32</v>
       </c>
       <c r="I7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K7" t="s">
         <v>36</v>
@@ -1497,7 +1497,7 @@
         <v>15</v>
       </c>
       <c r="E8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F8" t="s">
         <v>33</v>
@@ -1526,7 +1526,7 @@
         <v>15</v>
       </c>
       <c r="E9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F9" t="s">
         <v>79</v>
@@ -1584,7 +1584,7 @@
         <v>68</v>
       </c>
       <c r="I11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K11" t="s">
         <v>16</v>
@@ -1627,7 +1627,7 @@
         <v>50</v>
       </c>
       <c r="F13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I13" t="s">
         <v>48</v>
@@ -1751,7 +1751,7 @@
         <v>95</v>
       </c>
       <c r="B18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C18" t="s">
         <v>15</v>
@@ -1760,7 +1760,7 @@
         <v>43</v>
       </c>
       <c r="F18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I18" t="s">
         <v>35</v>
@@ -1777,19 +1777,19 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" t="s">
         <v>106</v>
-      </c>
-      <c r="B19" t="s">
-        <v>107</v>
       </c>
       <c r="C19" t="s">
         <v>15</v>
       </c>
       <c r="E19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I19" t="s">
         <v>35</v>
@@ -1806,19 +1806,19 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>114</v>
+      </c>
+      <c r="B20" t="s">
         <v>115</v>
-      </c>
-      <c r="B20" t="s">
-        <v>116</v>
       </c>
       <c r="C20" t="s">
         <v>15</v>
       </c>
       <c r="E20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F20" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J20" t="s">
         <v>34</v>
@@ -1829,22 +1829,22 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
+        <v>114</v>
+      </c>
+      <c r="B21" t="s">
         <v>115</v>
-      </c>
-      <c r="B21" t="s">
-        <v>116</v>
       </c>
       <c r="C21" t="s">
         <v>15</v>
       </c>
       <c r="E21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F21" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J21" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L21" t="s">
         <v>34</v>
@@ -1867,7 +1867,7 @@
         <v>85</v>
       </c>
       <c r="I22" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J22" t="s">
         <v>34</v>
@@ -2009,13 +2009,13 @@
         <v>43</v>
       </c>
       <c r="F27" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I27" t="s">
         <v>35</v>
       </c>
       <c r="J27" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K27" t="s">
         <v>36</v>
@@ -2096,13 +2096,13 @@
         <v>43</v>
       </c>
       <c r="F30" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I30" t="s">
         <v>69</v>
       </c>
       <c r="J30" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K30" t="s">
         <v>36</v>
@@ -2122,7 +2122,7 @@
         <v>42</v>
       </c>
       <c r="E31" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F31" t="s">
         <v>64</v>
@@ -2151,10 +2151,10 @@
         <v>42</v>
       </c>
       <c r="E32" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F32" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I32" t="s">
         <v>86</v>
@@ -2180,7 +2180,7 @@
         <v>42</v>
       </c>
       <c r="E33" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F33" t="s">
         <v>39</v>
@@ -2223,7 +2223,7 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B35" t="s">
         <v>58</v>
@@ -2232,10 +2232,10 @@
         <v>15</v>
       </c>
       <c r="E35" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I35" t="s">
         <v>37</v>
@@ -2249,7 +2249,7 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B36" t="s">
         <v>60</v>
@@ -2261,10 +2261,10 @@
         <v>53</v>
       </c>
       <c r="F36" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G36" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I36" t="s">
         <v>30</v>
@@ -2290,7 +2290,7 @@
         <v>62</v>
       </c>
       <c r="G37" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K37" t="s">
         <v>36</v>
@@ -2301,7 +2301,7 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B38" t="s">
         <v>60</v>
@@ -2313,13 +2313,13 @@
         <v>43</v>
       </c>
       <c r="F38" t="s">
+        <v>122</v>
+      </c>
+      <c r="G38" t="s">
+        <v>101</v>
+      </c>
+      <c r="I38" t="s">
         <v>123</v>
-      </c>
-      <c r="G38" t="s">
-        <v>102</v>
-      </c>
-      <c r="I38" t="s">
-        <v>124</v>
       </c>
       <c r="J38" t="s">
         <v>48</v>
@@ -2371,7 +2371,7 @@
         <v>17</v>
       </c>
       <c r="E40" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F40" t="s">
         <v>56</v>
@@ -2391,10 +2391,10 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B41" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C41" t="s">
         <v>17</v>
@@ -2403,10 +2403,10 @@
         <v>50</v>
       </c>
       <c r="F41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G41" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I41" t="s">
         <v>74</v>
@@ -2417,10 +2417,10 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B42" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C42" t="s">
         <v>17</v>
@@ -2429,10 +2429,10 @@
         <v>50</v>
       </c>
       <c r="F42" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G42" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I42" t="s">
         <v>80</v>
@@ -2443,42 +2443,42 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
+        <v>132</v>
+      </c>
+      <c r="B43" t="s">
         <v>133</v>
-      </c>
-      <c r="B43" t="s">
-        <v>134</v>
       </c>
       <c r="C43" t="s">
         <v>15</v>
       </c>
       <c r="E43" t="s">
+        <v>134</v>
+      </c>
+      <c r="F43" t="s">
         <v>135</v>
       </c>
-      <c r="F43" t="s">
-        <v>136</v>
-      </c>
       <c r="N43" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
+        <v>132</v>
+      </c>
+      <c r="B44" t="s">
         <v>133</v>
-      </c>
-      <c r="B44" t="s">
-        <v>134</v>
       </c>
       <c r="C44" t="s">
         <v>15</v>
       </c>
       <c r="E44" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F44" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Validate trades and support Split_sectors parsing
Add consistency checks and parsing support for the Split_sectors model and add a new model settings file. Introduces model_settings_eq.xlsx for the model with equalities, while the standard is with inequalities.
Adjust _cvxlab_results_parser_split_sectors to subtract new-sector V values from the parent sector.
Add trade-data validation that raises on inconsistencies (trade > parent Z+Y), zero out within-region trades to avoid issues.
</commit_message>
<xml_diff>
--- a/mario/tools/cvxlab/Split_sectors/model_settings.xlsx
+++ b/mario/tools/cvxlab/Split_sectors/model_settings.xlsx
@@ -5,16 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enextgen22.sharepoint.com/sites/entice/Shared Documents/WPs, Tasks &amp; Deliverables/WP2 - Data/T2.2 &amp; T2.3 - GTAP disaggregation/Disaggregation/MARIO implementation examples/2r 2s smallest/cvxlab test - new ob fun/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/tools/cvxlab/Split_sectors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{A4FE0614-723F-4058-911D-2BAED614CEC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{879EC62E-9443-4E4E-A867-B8810AFE3A09}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{0BD29A10-27A8-41FD-81E1-A0312648E109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EF126AB-6E0A-4569-9649-9721F3141D61}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="820" windowWidth="19250" windowHeight="11180" xr2:uid="{5885115D-3BA4-42C5-A7B9-D2CCF4E386B9}"/>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
+    <workbookView xWindow="120" yWindow="-14820" windowWidth="14400" windowHeight="10660" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
   </bookViews>
   <sheets>
-    <sheet name="problem" sheetId="5" r:id="rId1"/>
+    <sheet name="problem" sheetId="8" r:id="rId1"/>
     <sheet name="structure_sets" sheetId="1" r:id="rId2"/>
     <sheet name="structure_variables" sheetId="7" r:id="rId3"/>
   </sheets>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="152">
   <si>
     <t>set_key</t>
   </si>
@@ -248,18 +247,6 @@
     <t>Znew_supply</t>
   </si>
   <si>
-    <t>Constraint 1a(Z):  total consumption consistency by region and sector (excl. parent/new) before and after the new sector addition</t>
-  </si>
-  <si>
-    <t>Constraint 1a(Y):  total consumption consistency by region and sector (excl. parent/new) before and after the new sector addition</t>
-  </si>
-  <si>
-    <t>Constraint 1b:  total consumption consistency by region and sector (only parent/new supply) before and after the new sector addition</t>
-  </si>
-  <si>
-    <t>Constraint 1c:  total consumption consistency by region and sector (parent/new use of stables) before and after the new sector addition</t>
-  </si>
-  <si>
     <t>set1and2_to_set1</t>
   </si>
   <si>
@@ -320,9 +307,6 @@
     <t>sector_from,region_from, region_to</t>
   </si>
   <si>
-    <t>Constraint 4: trade balance</t>
-  </si>
-  <si>
     <t>Znew_use_pn_pn</t>
   </si>
   <si>
@@ -347,27 +331,9 @@
     <t>New total production</t>
   </si>
   <si>
-    <t>Constraint 3: column sum (Avoid redundancy, keep only for new)</t>
-  </si>
-  <si>
-    <t>Zold_p_st == I_p_r_from_to @ block_diag(I_p_pn,regions) @ Znew_supply</t>
-  </si>
-  <si>
-    <t>Yold_p ==  I_p_r_from_to @ block_diag(I_p_pn,regions) @ Ynew_pn</t>
-  </si>
-  <si>
-    <t>Zold_p_p == I_p_r_from_to @ block_diag(I_p_pn,regions) @ Znew_use_pn_pn @ tran(block_diag(I_p_pn,regions)) @ I_p_r_from_to</t>
-  </si>
-  <si>
-    <t>Zold_st_p ==  Znew_use_st_pn @ tran(block_diag(I_p_pn,regions)) @ I_p_r_from_to</t>
-  </si>
-  <si>
     <t>I_col</t>
   </si>
   <si>
-    <t>Constraint 2: total production of parent and new sectors = total consumption of their outputs</t>
-  </si>
-  <si>
     <t>I_r_st</t>
   </si>
   <si>
@@ -395,12 +361,6 @@
     <t>region_to, cons_categ</t>
   </si>
   <si>
-    <t>Xnew_pn==Znew_supply@I_r_st+Znew_use_pn_pn@I_r_pn+Ynew_pn@I_r_c</t>
-  </si>
-  <si>
-    <t>tran(I_rs_from_to_n@Xnew_n) ==I_col @ Znew_use_n + VA_n</t>
-  </si>
-  <si>
     <t>tol</t>
   </si>
   <si>
@@ -434,9 +394,6 @@
     <t>I_rpn_r</t>
   </si>
   <si>
-    <t>Trade == mult(Znew_supply_imp @ I_rst_r @ I_r_from_to, Trade_selector) + mult(Znew_use_pn_pn_imp@ I_rpn_r @ I_r_from_to, Trade_selector) + mult(Ynew_imp @ I_rc_r @ I_r_from_to, Trade_selector)</t>
-  </si>
-  <si>
     <t>Znew_use_pn_pn_imp</t>
   </si>
   <si>
@@ -453,6 +410,90 @@
   </si>
   <si>
     <t>nonneg</t>
+  </si>
+  <si>
+    <t>Zold_p_p &gt;= (I_p_r_from_to @ block_diag(I_p_pn,regions) @ Znew_use_pn_pn @ tran(block_diag(I_p_pn,regions)) @ I_p_r_from_to)*(1-eps)</t>
+  </si>
+  <si>
+    <t>Zold_p_p &lt;= (I_p_r_from_to @ block_diag(I_p_pn,regions) @ Znew_use_pn_pn @ tran(block_diag(I_p_pn,regions)) @ I_p_r_from_to)*(1+eps)</t>
+  </si>
+  <si>
+    <t>Zold_p_st &gt;=( I_p_r_from_to @ block_diag(I_p_pn,regions) @ Znew_supply)*(1-eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Z)+:  total consumption consistency by region and sector (excl. parent/new) before and after the new sector addition</t>
+  </si>
+  <si>
+    <t>Zold_p_st &lt;=( I_p_r_from_to @ block_diag(I_p_pn,regions) @ Znew_supply)*(1+eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Z)-:  total consumption consistency by region and sector (excl. parent/new) before and after the new sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Y)-:  total consumption consistency by region and sector (excl. parent/new) before and after the new sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Y)+:  total consumption consistency by region and sector (excl. parent/new) before and after the new sector addition</t>
+  </si>
+  <si>
+    <t>Yold_p &gt;= ( I_p_r_from_to @ block_diag(I_p_pn,regions) @ Ynew_pn)*(1-eps)</t>
+  </si>
+  <si>
+    <t>Yold_p &lt;= ( I_p_r_from_to @ block_diag(I_p_pn,regions) @ Ynew_pn)*(1+eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1b-:  total consumption consistency by region and sector (only parent/new supply) before and after the new sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1b+:  total consumption consistency by region and sector (only parent/new supply) before and after the new sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1c-:  total consumption consistency by region and sector (parent/new use of stables) before and after the new sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1c+:  total consumption consistency by region and sector (parent/new use of stables) before and after the new sector addition</t>
+  </si>
+  <si>
+    <t>Zold_st_p &gt;=  (Znew_use_st_pn @ tran(block_diag(I_p_pn,regions)) @ I_p_r_from_to)*(1-eps)</t>
+  </si>
+  <si>
+    <t>Zold_st_p &lt;=  (Znew_use_st_pn @ tran(block_diag(I_p_pn,regions)) @ I_p_r_from_to)*(1+eps)</t>
+  </si>
+  <si>
+    <t>Xnew_pn&gt;=(Znew_supply@I_r_st+Znew_use_pn_pn@I_r_pn+Ynew_pn@I_r_c)*(1-eps)</t>
+  </si>
+  <si>
+    <t>Constraint 2-: total production of parent and new sectors = total consumption of their outputs</t>
+  </si>
+  <si>
+    <t>Xnew_pn&lt;=(Znew_supply@I_r_st+Znew_use_pn_pn@I_r_pn+Ynew_pn@I_r_c)*(1+eps)</t>
+  </si>
+  <si>
+    <t>Constraint 3-: column sum (Avoid redundancy, keep only for new)</t>
+  </si>
+  <si>
+    <t>Constraint 2+: total production of parent and new sectors = total consumption of their outputs</t>
+  </si>
+  <si>
+    <t>Constraint 3+: column sum (Avoid redundancy, keep only for new)</t>
+  </si>
+  <si>
+    <t>Constraint 4-: trade balance</t>
+  </si>
+  <si>
+    <t>Constraint 4+: trade balance</t>
+  </si>
+  <si>
+    <t>tran(I_rs_from_to_n@Xnew_n) &gt;= (I_col @ Znew_use_n + VA_n) * (1-delta)</t>
+  </si>
+  <si>
+    <t>tran(I_rs_from_to_n@Xnew_n) &lt;= (I_col @ Znew_use_n + VA_n) * (1+delta)</t>
+  </si>
+  <si>
+    <t>Trade &gt;= (mult(Znew_supply_imp @ I_rst_r @ I_r_from_to, Trade_selector) + mult(Znew_use_pn_pn_imp@ I_rpn_r @ I_r_from_to, Trade_selector) + mult(Ynew_imp @ I_rc_r @ I_r_from_to, Trade_selector)) *(1-delta)</t>
+  </si>
+  <si>
+    <t>Trade &lt;= (mult(Znew_supply_imp @ I_rst_r @ I_r_from_to, Trade_selector) + mult(Znew_use_pn_pn_imp@ I_rpn_r @ I_r_from_to, Trade_selector) + mult(Ynew_imp @ I_rc_r @ I_r_from_to, Trade_selector)) *(1+delta)</t>
   </si>
 </sst>
 </file>
@@ -560,7 +601,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -575,9 +616,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -879,8 +917,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18E309D5-3CF9-4805-9054-67D3EBAC901C}">
-  <dimension ref="A1:D10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A04F280-5EF4-412D-AFEE-E04537690E44}">
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
@@ -905,68 +943,120 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>69</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>70</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
-        <v>105</v>
+        <v>132</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>72</v>
+        <v>133</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C8" s="7" t="s">
-        <v>119</v>
+      <c r="C8" t="s">
+        <v>125</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C9" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C10" s="6"/>
-      <c r="D10" s="5"/>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C9" t="s">
+        <v>138</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C11" t="s">
+        <v>140</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C12" t="s">
+        <v>142</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C13" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C14" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C15" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C16" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>147</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1009,7 +1099,7 @@
         <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -1020,7 +1110,7 @@
         <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -1041,7 +1131,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B6" t="s">
         <v>25</v>
@@ -1049,13 +1139,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="E7" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1106,8 +1196,8 @@
       <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="10" t="s">
-        <v>137</v>
+      <c r="I1" s="3" t="s">
+        <v>123</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>21</v>
@@ -1122,10 +1212,10 @@
         <v>24</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
@@ -1226,7 +1316,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>32</v>
@@ -1249,7 +1339,7 @@
         <v>58</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>15</v>
@@ -1272,7 +1362,7 @@
         <v>58</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>15</v>
@@ -1281,7 +1371,7 @@
         <v>47</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>46</v>
@@ -1292,22 +1382,22 @@
     </row>
     <row r="8" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="M8" s="9" t="s">
         <v>33</v>
@@ -1341,10 +1431,10 @@
     </row>
     <row r="10" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>15</v>
@@ -1353,13 +1443,13 @@
         <v>42</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>35</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="L10" s="9" t="s">
         <v>35</v>
@@ -1370,10 +1460,10 @@
     </row>
     <row r="11" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>15</v>
@@ -1382,7 +1472,7 @@
         <v>42</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>60</v>
@@ -1402,7 +1492,7 @@
         <v>65</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1411,7 +1501,7 @@
         <v>42</v>
       </c>
       <c r="F12" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="I12" t="b">
         <v>1</v>
@@ -1434,7 +1524,7 @@
         <v>65</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -1443,7 +1533,7 @@
         <v>42</v>
       </c>
       <c r="F13" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I13" t="b">
         <v>1</v>
@@ -1452,7 +1542,7 @@
         <v>35</v>
       </c>
       <c r="K13" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="L13" t="s">
         <v>35</v>
@@ -1466,7 +1556,7 @@
         <v>65</v>
       </c>
       <c r="B14" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C14" t="s">
         <v>41</v>
@@ -1476,7 +1566,7 @@
         <v>42</v>
       </c>
       <c r="F14" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="G14"/>
       <c r="H14"/>
@@ -1484,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="K14" t="s">
         <v>66</v>
@@ -1504,7 +1594,7 @@
         <v>65</v>
       </c>
       <c r="B15" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
         <v>41</v>
@@ -1514,7 +1604,7 @@
         <v>42</v>
       </c>
       <c r="F15" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="G15"/>
       <c r="H15"/>
@@ -1542,7 +1632,7 @@
         <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
         <v>41</v>
@@ -1580,7 +1670,7 @@
         <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C17" t="s">
         <v>41</v>
@@ -1618,7 +1708,7 @@
         <v>68</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
         <v>41</v>
@@ -1657,7 +1747,7 @@
       </c>
       <c r="D19"/>
       <c r="E19" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F19" t="s">
         <v>57</v>
@@ -1694,7 +1784,7 @@
         <v>41</v>
       </c>
       <c r="E20" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F20" t="s">
         <v>38</v>
@@ -1717,7 +1807,7 @@
     </row>
     <row r="21" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B21" s="8" t="s">
         <v>53</v>
@@ -1729,10 +1819,10 @@
         <v>42</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="J21" s="8" t="s">
         <v>29</v>
@@ -1749,10 +1839,10 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>16</v>
@@ -1762,10 +1852,10 @@
         <v>23</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="H22" s="8"/>
       <c r="I22" s="8"/>
@@ -1776,7 +1866,7 @@
     </row>
     <row r="23" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>53</v>
@@ -1788,13 +1878,13 @@
         <v>42</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="K23" s="8" t="s">
         <v>46</v>
@@ -1808,10 +1898,10 @@
     </row>
     <row r="24" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="8" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>16</v>
@@ -1820,10 +1910,10 @@
         <v>47</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="J24" s="8" t="s">
         <v>33</v>
@@ -1834,22 +1924,22 @@
     </row>
     <row r="25" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="8" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="K25" s="8" t="s">
         <v>60</v>
@@ -1860,22 +1950,22 @@
     </row>
     <row r="26" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="K26" s="8" t="s">
         <v>34</v>
@@ -1886,22 +1976,22 @@
     </row>
     <row r="27" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="M27" s="8" t="s">
         <v>35</v>
@@ -1912,7 +2002,7 @@
     </row>
     <row r="28" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="B28" s="8" t="s">
         <v>49</v>
@@ -1924,10 +2014,10 @@
         <v>56</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K28" s="8" t="s">
         <v>60</v>
@@ -1941,7 +2031,7 @@
     </row>
     <row r="29" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="B29" s="8" t="s">
         <v>49</v>
@@ -1953,10 +2043,10 @@
         <v>56</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K29" s="8" t="s">
         <v>34</v>
@@ -1970,7 +2060,7 @@
     </row>
     <row r="30" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="B30" s="8" t="s">
         <v>50</v>
@@ -1979,13 +2069,13 @@
         <v>16</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="L30" s="8" t="s">
         <v>33</v>
@@ -2014,7 +2104,7 @@
         <v>55</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="L31" s="8" t="s">
         <v>35</v>
@@ -2025,7 +2115,7 @@
     </row>
     <row r="32" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="9" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B32" s="9" t="s">
         <v>51</v>
@@ -2034,10 +2124,10 @@
         <v>15</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="J32" s="9" t="s">
         <v>36</v>
@@ -2051,7 +2141,7 @@
     </row>
     <row r="33" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="9" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B33" s="9" t="s">
         <v>48</v>
@@ -2063,7 +2153,7 @@
         <v>54</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="J33" s="9" t="s">
         <v>66</v>
@@ -2074,42 +2164,42 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="B34" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="C34" t="s">
         <v>15</v>
       </c>
       <c r="E34" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="F34" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="O34" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="B35" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="C35" t="s">
         <v>15</v>
       </c>
       <c r="E35" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="F35" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="O35" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -2119,8 +2209,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="348072715f26cde881c56d84fe7c6dcc">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="53f9bc5e977a2cc0a870214cffd63ac6" ns2:_="" ns3:_="">
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="90e7079a-7589-470d-892b-836f3f5ab9a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9ef6bf99-292f-445d-95df-6a8984d5eb85" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="3916dc5588df290b35e5c499b507bc33">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e3fae628afbc47c424dc6703fd07071" ns2:_="" ns3:_="">
     <xsd:import namespace="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
     <xsd:import namespace="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
     <xsd:element name="properties">
@@ -2169,7 +2279,7 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Tag immagine" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -2223,8 +2333,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo di contenuto"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titolo"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -2313,46 +2423,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="90e7079a-7589-470d-892b-836f3f5ab9a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9ef6bf99-292f-445d-95df-6a8984d5eb85" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D79060E-3E34-464E-B404-C7C8F25066D5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
-    <ds:schemaRef ds:uri="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6344D8B-6291-40EE-A141-20586EBB6785}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -2369,10 +2440,29 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91788BB2-4A3F-4B3D-BB9A-4A497CBAE5D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2A1479F-B33D-4F74-85D6-829DDA2D4620}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
+    <ds:schemaRef ds:uri="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fixing creation of input data for Split sector cvxlab problem
Setting in all tables the values <1e-6 to 0.
Automatically set to 0 in Trade_selector when same r_to e r_from
</commit_message>
<xml_diff>
--- a/mario/tools/cvxlab/Split_sectors/model_settings.xlsx
+++ b/mario/tools/cvxlab/Split_sectors/model_settings.xlsx
@@ -1,17 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/tools/cvxlab/Split_sectors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="8_{A4FE0614-723F-4058-911D-2BAED614CEC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8637C9D-3149-46A0-A857-061B405C02C1}"/>
+  <xr:revisionPtr revIDLastSave="263" documentId="8_{A50511BF-6CF0-4AF4-AD61-47C0180FA04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90A83F41-3413-4019-BAFF-1512FFAB6694}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5885115D-3BA4-42C5-A7B9-D2CCF4E386B9}"/>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
+    <workbookView xWindow="-60" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="657" xr2:uid="{ADE65AC1-7326-4C1C-AEEF-E9867C94CCED}"/>
   </bookViews>
   <sheets>
     <sheet name="problem" sheetId="5" r:id="rId1"/>
@@ -19,7 +18,7 @@
     <sheet name="structure_variables" sheetId="7" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">structure_variables!$A$1:$N$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">structure_variables!$A$1:$N$30</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="172">
   <si>
     <t>set_key</t>
   </si>
@@ -137,9 +136,6 @@
     <t>Yold</t>
   </si>
   <si>
-    <t>Yold_p</t>
-  </si>
-  <si>
     <t>dim: cols</t>
   </si>
   <si>
@@ -173,9 +169,6 @@
     <t>region_from, region_to, sector_from</t>
   </si>
   <si>
-    <t>dim: rows, filters: {category: [new]}</t>
-  </si>
-  <si>
     <t>region_from, sector_from</t>
   </si>
   <si>
@@ -221,18 +214,6 @@
     <t>dim: cols, filters: {category: [parent, new]}</t>
   </si>
   <si>
-    <t>Constraint 1a(Z):  total consumption consistency by region and sector (excl. parent/new) before and after the new sector addition</t>
-  </si>
-  <si>
-    <t>Constraint 1a(Y):  total consumption consistency by region and sector (excl. parent/new) before and after the new sector addition</t>
-  </si>
-  <si>
-    <t>Constraint 1b:  total consumption consistency by region and sector (only parent/new supply) before and after the new sector addition</t>
-  </si>
-  <si>
-    <t>Constraint 1c:  total consumption consistency by region and sector (parent/new use of stables) before and after the new sector addition</t>
-  </si>
-  <si>
     <t>set1and2_to_set1</t>
   </si>
   <si>
@@ -257,9 +238,6 @@
     <t>category: [stable, parent, new]</t>
   </si>
   <si>
-    <t>I_rs_from_to_n</t>
-  </si>
-  <si>
     <t>dim: cols, filters: {category: [new]}</t>
   </si>
   <si>
@@ -278,211 +256,304 @@
     <t>sector_from,region_from, region_to</t>
   </si>
   <si>
-    <t>Constraint 4: trade balance</t>
-  </si>
-  <si>
     <t>I_p_pn</t>
   </si>
   <si>
+    <t>regions</t>
+  </si>
+  <si>
+    <t>Length of regions set</t>
+  </si>
+  <si>
+    <t>set_length</t>
+  </si>
+  <si>
+    <t>dim: rows, filters: {category: [parent,new]}</t>
+  </si>
+  <si>
+    <t>New total production</t>
+  </si>
+  <si>
+    <t>I_r_st</t>
+  </si>
+  <si>
+    <t>Col vector as long as regions and stable sectors</t>
+  </si>
+  <si>
+    <t>Row vector as long as regions and sectors</t>
+  </si>
+  <si>
+    <t>I_r_pn</t>
+  </si>
+  <si>
+    <t>Col vector as long as regions and parent-new sectors</t>
+  </si>
+  <si>
+    <t>I_rc_r</t>
+  </si>
+  <si>
+    <t>I_r_c</t>
+  </si>
+  <si>
+    <t>Col vector as long as regions and consumption categories</t>
+  </si>
+  <si>
+    <t>region_to, cons_categ</t>
+  </si>
+  <si>
+    <t>tol</t>
+  </si>
+  <si>
+    <t>Tolerance scalars</t>
+  </si>
+  <si>
+    <t>scalar</t>
+  </si>
+  <si>
+    <t>delta</t>
+  </si>
+  <si>
+    <t>dim: rows, filters: {tolerance: delta}</t>
+  </si>
+  <si>
+    <t>eps</t>
+  </si>
+  <si>
+    <t>dim: rows, filters: {tolerance: eps}</t>
+  </si>
+  <si>
+    <t>Single item for defining scalars</t>
+  </si>
+  <si>
+    <t>tolerance: [delta,eps]</t>
+  </si>
+  <si>
+    <t>I_rst_r</t>
+  </si>
+  <si>
+    <t>I_rpn_r</t>
+  </si>
+  <si>
+    <t>nonneg</t>
+  </si>
+  <si>
+    <t>dim: intra</t>
+  </si>
+  <si>
+    <t>New total production (r_to,s_to)</t>
+  </si>
+  <si>
+    <t>Constraint 3b: auxiliary matrix for column sum</t>
+  </si>
+  <si>
+    <t>Z0</t>
+  </si>
+  <si>
+    <t>Z0_all_n</t>
+  </si>
+  <si>
+    <t>Z0_st_p</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>XT</t>
+  </si>
+  <si>
+    <t>XT_intra</t>
+  </si>
+  <si>
+    <t>Z_use</t>
+  </si>
+  <si>
+    <t>Z_use_st_p</t>
+  </si>
+  <si>
+    <t>Z_use_n</t>
+  </si>
+  <si>
+    <t>Z_use_pn_pn_to</t>
+  </si>
+  <si>
+    <t>Z_use_pn_pn_from</t>
+  </si>
+  <si>
+    <t>Z_use_st_pn</t>
+  </si>
+  <si>
+    <t>Z_supply</t>
+  </si>
+  <si>
+    <t>Z_supply_to</t>
+  </si>
+  <si>
+    <t>Z_supply_from</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Y_pn_to</t>
+  </si>
+  <si>
+    <t>Y_pn_from</t>
+  </si>
+  <si>
+    <t>Y_imp</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>factor, region_to, sector_to</t>
+  </si>
+  <si>
+    <t>dim: cols, filters: {category: [parent,new]}</t>
+  </si>
+  <si>
+    <t>factor</t>
+  </si>
+  <si>
+    <t>I_row_v</t>
+  </si>
+  <si>
+    <t>Row vector as long as factors of production</t>
+  </si>
+  <si>
+    <t>I_row_rs</t>
+  </si>
+  <si>
+    <t>Vold</t>
+  </si>
+  <si>
+    <t>V0</t>
+  </si>
+  <si>
+    <t>Factors of production (rows of V)</t>
+  </si>
+  <si>
     <t>I_p_r_from_to</t>
   </si>
   <si>
-    <t>regions</t>
-  </si>
-  <si>
-    <t>Length of regions set</t>
-  </si>
-  <si>
-    <t>set_length</t>
-  </si>
-  <si>
-    <t>dim: rows, filters: {category: [parent,new]}</t>
-  </si>
-  <si>
-    <t>New total production</t>
-  </si>
-  <si>
-    <t>Constraint 3: column sum (Avoid redundancy, keep only for new)</t>
-  </si>
-  <si>
-    <t>Constraint 2: total production of parent and new sectors = total consumption of their outputs</t>
-  </si>
-  <si>
-    <t>I_r_st</t>
-  </si>
-  <si>
-    <t>Col vector as long as regions and stable sectors</t>
-  </si>
-  <si>
-    <t>Row vector as long as regions and sectors</t>
-  </si>
-  <si>
-    <t>I_r_pn</t>
-  </si>
-  <si>
-    <t>Col vector as long as regions and parent-new sectors</t>
-  </si>
-  <si>
-    <t>I_rc_r</t>
-  </si>
-  <si>
-    <t>I_r_c</t>
-  </si>
-  <si>
-    <t>Col vector as long as regions and consumption categories</t>
-  </si>
-  <si>
-    <t>region_to, cons_categ</t>
-  </si>
-  <si>
-    <t>tol</t>
-  </si>
-  <si>
-    <t>Tolerance scalars</t>
-  </si>
-  <si>
-    <t>scalar</t>
-  </si>
-  <si>
-    <t>delta</t>
-  </si>
-  <si>
-    <t>dim: rows, filters: {tolerance: delta}</t>
-  </si>
-  <si>
-    <t>eps</t>
-  </si>
-  <si>
-    <t>dim: rows, filters: {tolerance: eps}</t>
-  </si>
-  <si>
-    <t>Single item for defining scalars</t>
-  </si>
-  <si>
-    <t>tolerance: [delta,eps]</t>
-  </si>
-  <si>
-    <t>I_rst_r</t>
-  </si>
-  <si>
-    <t>I_rpn_r</t>
-  </si>
-  <si>
-    <t>nonneg</t>
-  </si>
-  <si>
-    <t>Vold == V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to)</t>
-  </si>
-  <si>
-    <t>Constraint 5: VA consistency</t>
-  </si>
-  <si>
-    <t>factor</t>
-  </si>
-  <si>
-    <t>Factors of production (rows of V)</t>
-  </si>
-  <si>
-    <t>Vold</t>
-  </si>
-  <si>
-    <t>V0</t>
-  </si>
-  <si>
-    <t>X_pn</t>
-  </si>
-  <si>
-    <t>X_n</t>
-  </si>
-  <si>
-    <t>Z0_all_n</t>
-  </si>
-  <si>
-    <t>Z0_st_p</t>
-  </si>
-  <si>
-    <t>Z_use_st_p</t>
-  </si>
-  <si>
-    <t>Z_use_n</t>
-  </si>
-  <si>
-    <t>Z_use_pn_pn</t>
-  </si>
-  <si>
-    <t>Z_use_pn_pn_imp</t>
-  </si>
-  <si>
-    <t>Z_use_st_pn</t>
-  </si>
-  <si>
-    <t>Z_supply</t>
-  </si>
-  <si>
-    <t>Z_supply_imp</t>
-  </si>
-  <si>
-    <t>Y_pn</t>
-  </si>
-  <si>
-    <t>Y_imp</t>
-  </si>
-  <si>
-    <t>V</t>
-  </si>
-  <si>
-    <t>dim: cols, filters: {category: [parent,new]}</t>
-  </si>
-  <si>
-    <t>V_n</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>Z0</t>
-  </si>
-  <si>
-    <t>Z_use</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>factor, region_to, sector_to</t>
+    <t>Constraint 2+: total production of parent and  sectors = total consumption of their outputs</t>
+  </si>
+  <si>
+    <t>Constraint 2-: total production of parent and  sectors = total consumption of their outputs</t>
+  </si>
+  <si>
+    <t>Constraint 3a-: column sum (Avoid redundancy, keep only for )</t>
+  </si>
+  <si>
+    <t>Constraint 3a+: column sum (Avoid redundancy, keep only for )</t>
+  </si>
+  <si>
+    <t>Constraint 4+: trade balance</t>
+  </si>
+  <si>
+    <t>Constraint 4-: trade balance</t>
+  </si>
+  <si>
+    <t>Vold &gt;= (V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))*(1-delta)</t>
+  </si>
+  <si>
+    <t>Vold &lt;= (V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))*(1+delta)</t>
+  </si>
+  <si>
+    <t>Zold_p_st &lt;= (block_diag(I_p_pn,regions) @ Z_supply_to)*(1+eps)</t>
+  </si>
+  <si>
+    <t>Zold_p_st &gt;= (block_diag(I_p_pn,regions) @ Z_supply_to)*(1-eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Z)+:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Z)-:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Y)+:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1a(Y)-:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Zold_p_p &lt;= (block_diag(I_p_pn,regions) @ Z_use_pn_pn_to @ tran(I_p_pn))*(1+eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1b+:  total consumption consistency by region and sector (only parent/ supply) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1b-:  total consumption consistency by region and sector (only parent/ supply) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Zold_p_p &gt;= (block_diag(I_p_pn,regions) @ Z_use_pn_pn_to @ tran(I_p_pn))*(1-eps)</t>
+  </si>
+  <si>
+    <t>Zold_st_p &lt;= ( Z_use_st_pn @ tran(I_p_pn))*(1+eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1c+:  total consumption consistency by region and sector (parent/ use of stables) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Constraint 1c-:  total consumption consistency by region and sector (parent/ use of stables) before and after the  sector addition</t>
+  </si>
+  <si>
+    <t>Zold_st_p &gt;= ( Z_use_st_pn @ tran(I_p_pn))*(1-eps)</t>
+  </si>
+  <si>
+    <t>Z_use_n_pn</t>
+  </si>
+  <si>
+    <t>Z_supply_n</t>
+  </si>
+  <si>
+    <t>Trade &lt;= (mult(Z_supply_n @ I_rst_r @ I_r_from_to, Trade_selector) + mult(Z_use_n_pn@ I_rpn_r @ I_r_from_to, Trade_selector) + mult(Y_imp @ I_rc_r @ I_r_from_to, Trade_selector))*(1+delta)</t>
+  </si>
+  <si>
+    <t>Trade &gt;= (mult(Z_supply_n @ I_rst_r @ I_r_from_to, Trade_selector) + mult(Z_use_n_pn@ I_rpn_r @ I_r_from_to, Trade_selector) + mult(Y_imp @ I_rc_r @ I_r_from_to, Trade_selector))*(1-delta)</t>
+  </si>
+  <si>
+    <t>Yold &lt;= (block_diag(I_p_pn,regions) @ Y_pn_to)*(1+eps)</t>
+  </si>
+  <si>
+    <t>Yold &gt;= (block_diag(I_p_pn,regions) @ Y_pn_to)*(1-eps)</t>
+  </si>
+  <si>
+    <t>Constraint 1d+: VA consistency</t>
+  </si>
+  <si>
+    <t>Constraint 1d-: VA consistency</t>
+  </si>
+  <si>
+    <t>Z_use_to</t>
+  </si>
+  <si>
+    <t>V_intra</t>
+  </si>
+  <si>
+    <t>X_intra</t>
+  </si>
+  <si>
+    <t>I_rs_from_to_pn</t>
+  </si>
+  <si>
+    <t>XT_intra &gt;=(I_row_rs @ Z_use_to + I_row_v @ V_intra)*(1-delta)</t>
+  </si>
+  <si>
+    <t>XT_intra &lt;=(I_row_rs @ Z_use_to + I_row_v @ V_intra)*(1+delta)</t>
   </si>
   <si>
     <t>Minimize(sum(entropy(Z_use_n,Z0_all_n))+sum(entropy(Z_use_st_p,Z0_st_p))+sum(entropy(V,V0)))</t>
   </si>
   <si>
-    <t>Row vector as long as factors of production</t>
-  </si>
-  <si>
-    <t>I_row_rs</t>
-  </si>
-  <si>
-    <t>I_row_v</t>
-  </si>
-  <si>
-    <t>Zold_p_st == I_p_r_from_to @ block_diag(I_p_pn,regions) @ Z_supply</t>
-  </si>
-  <si>
-    <t>Zold_p_p == I_p_r_from_to @ block_diag(I_p_pn,regions) @ Z_use_pn_pn @ tran(block_diag(I_p_pn,regions)) @ I_p_r_from_to</t>
-  </si>
-  <si>
-    <t>Zold_st_p ==  Z_use_st_pn @ tran(block_diag(I_p_pn,regions)) @ I_p_r_from_to</t>
-  </si>
-  <si>
-    <t>Yold_p ==  I_p_r_from_to @ block_diag(I_p_pn,regions) @ Y_pn</t>
-  </si>
-  <si>
-    <t>Trade == mult(Z_supply_imp @ I_rst_r @ I_r_from_to, Trade_selector) + mult(Z_use_pn_pn_imp@ I_rpn_r @ I_r_from_to, Trade_selector) + mult(Y_imp @ I_rc_r @ I_r_from_to, Trade_selector)</t>
-  </si>
-  <si>
-    <t>X_pn==Z_supply@I_r_st+Z_use_pn_pn@I_r_pn+Y_pn@I_r_c</t>
-  </si>
-  <si>
-    <t>tran(I_rs_from_to_n@X_n) ==I_row_rs @ Z_use_n + I_row_v @ V_n</t>
+    <t>X_intra&lt;=(Z_supply_from@I_r_st+Z_use_pn_pn_from@I_r_pn+Y_pn_from@I_r_c)*(1+delta)</t>
+  </si>
+  <si>
+    <t>X_intra&gt;=(Z_supply_from@I_r_st+Z_use_pn_pn_from@I_r_pn+Y_pn_from@I_r_c)*(1-delta)</t>
+  </si>
+  <si>
+    <t>XT ==I_rs_from_to_pn @ X</t>
   </si>
 </sst>
 </file>
@@ -907,7 +978,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18E309D5-3CF9-4805-9054-67D3EBAC901C}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
@@ -932,39 +1003,39 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
-        <v>137</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>60</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>61</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
-        <v>143</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>63</v>
+        <v>159</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
@@ -972,31 +1043,103 @@
         <v>146</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>88</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C8" s="7" t="s">
-        <v>147</v>
+      <c r="C8" t="s">
+        <v>149</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C9" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="C10" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>111</v>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C10" t="s">
+        <v>153</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C11" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C12" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C13" t="s">
+        <v>169</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C14" t="s">
+        <v>170</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C15" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C16" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C17" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C18" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C19" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1040,7 +1183,7 @@
         <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -1051,7 +1194,7 @@
         <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -1072,7 +1215,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
         <v>25</v>
@@ -1080,21 +1223,21 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="B7" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="E8" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1104,7 +1247,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}">
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.26953125" customWidth="1"/>
@@ -1120,7 +1263,7 @@
     <col min="14" max="15" width="10.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
@@ -1146,7 +1289,7 @@
         <v>11</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>21</v>
@@ -1161,16 +1304,16 @@
         <v>24</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>26</v>
       </c>
@@ -1181,7 +1324,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -1190,16 +1333,16 @@
         <v>29</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>26</v>
       </c>
@@ -1210,7 +1353,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>30</v>
@@ -1219,16 +1362,16 @@
         <v>29</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>26</v>
       </c>
@@ -1239,478 +1382,438 @@
         <v>15</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J4" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="K4" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="K4" s="9" t="s">
-        <v>57</v>
-      </c>
       <c r="L4" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J5" s="9" t="s">
         <v>29</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M5" s="9" t="s">
-        <v>33</v>
+        <v>99</v>
       </c>
       <c r="N5" s="9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+      <c r="O6" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="O7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+      <c r="O7" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>132</v>
+        <v>40</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>86</v>
+        <v>41</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>116</v>
+        <v>40</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+      <c r="M8" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>132</v>
+        <v>102</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>44</v>
+        <v>34</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>66</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+      <c r="M9" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>41</v>
+        <v>102</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>36</v>
+        <v>53</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>55</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>133</v>
+        <v>105</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>118</v>
+        <v>164</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="M11" s="9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
-        <v>133</v>
+        <v>105</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="9"/>
       <c r="E12" s="9" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
+        <v>105</v>
+      </c>
       <c r="J12" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="K12" s="9" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="M12" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>134</v>
+        <v>106</v>
       </c>
       <c r="B13" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E13" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="F13" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="I13" t="b">
         <v>1</v>
       </c>
-      <c r="J13" t="s">
-        <v>55</v>
-      </c>
       <c r="K13" t="s">
-        <v>57</v>
-      </c>
-      <c r="L13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M13" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>134</v>
+        <v>106</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14"/>
+        <v>38</v>
+      </c>
       <c r="E14" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="F14" t="s">
-        <v>121</v>
-      </c>
-      <c r="G14"/>
-      <c r="H14"/>
+        <v>107</v>
+      </c>
       <c r="I14" t="b">
         <v>1</v>
       </c>
-      <c r="J14" t="s">
-        <v>35</v>
-      </c>
       <c r="K14" t="s">
-        <v>73</v>
-      </c>
-      <c r="L14" t="s">
-        <v>35</v>
+        <v>123</v>
       </c>
       <c r="M14" t="s">
-        <v>33</v>
-      </c>
-      <c r="N14"/>
-      <c r="O14"/>
-      <c r="P14"/>
-      <c r="Q14"/>
-    </row>
-    <row r="15" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" t="s">
         <v>39</v>
       </c>
-      <c r="D15"/>
-      <c r="E15" t="s">
-        <v>40</v>
-      </c>
       <c r="F15" t="s">
-        <v>122</v>
-      </c>
-      <c r="G15"/>
-      <c r="H15"/>
+        <v>109</v>
+      </c>
       <c r="I15" t="b">
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="K15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="L15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M15" t="s">
-        <v>33</v>
-      </c>
-      <c r="N15"/>
-      <c r="O15"/>
-      <c r="P15"/>
-      <c r="Q15"/>
-    </row>
-    <row r="16" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="B16" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C16" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" t="s">
         <v>39</v>
       </c>
-      <c r="D16"/>
-      <c r="E16" t="s">
-        <v>40</v>
-      </c>
       <c r="F16" t="s">
-        <v>123</v>
-      </c>
-      <c r="G16"/>
-      <c r="H16"/>
+        <v>110</v>
+      </c>
       <c r="I16" t="b">
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K16" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="L16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M16" t="s">
-        <v>33</v>
-      </c>
-      <c r="N16"/>
-      <c r="O16"/>
-      <c r="P16"/>
-      <c r="Q16"/>
-    </row>
-    <row r="17" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="B17" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" t="s">
         <v>39</v>
       </c>
-      <c r="D17"/>
-      <c r="E17" t="s">
-        <v>40</v>
-      </c>
       <c r="F17" t="s">
-        <v>124</v>
-      </c>
-      <c r="G17"/>
-      <c r="H17"/>
+        <v>162</v>
+      </c>
       <c r="I17" t="b">
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="K17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M17" t="s">
-        <v>33</v>
-      </c>
-      <c r="N17"/>
-      <c r="O17"/>
-      <c r="P17"/>
-      <c r="Q17"/>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18"/>
+      <c r="E18" t="s">
         <v>39</v>
       </c>
-      <c r="E18" t="s">
-        <v>40</v>
-      </c>
       <c r="F18" t="s">
-        <v>125</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="G18"/>
+      <c r="H18"/>
       <c r="I18" t="b">
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>34</v>
+        <v>76</v>
       </c>
       <c r="K18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M18" t="s">
-        <v>33</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="N18"/>
+      <c r="O18"/>
+      <c r="P18"/>
+      <c r="Q18"/>
     </row>
     <row r="19" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D19"/>
       <c r="E19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F19" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G19"/>
       <c r="H19"/>
@@ -1718,613 +1821,835 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="K19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L19" t="s">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="M19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N19"/>
       <c r="O19"/>
       <c r="P19"/>
       <c r="Q19"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="B20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" t="s">
         <v>38</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20"/>
+      <c r="E20" t="s">
         <v>39</v>
       </c>
-      <c r="E20" t="s">
-        <v>75</v>
-      </c>
       <c r="F20" t="s">
-        <v>127</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="G20"/>
+      <c r="H20"/>
       <c r="I20" t="b">
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="K20" t="s">
+        <v>57</v>
       </c>
       <c r="L20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M20" t="s">
-        <v>33</v>
-      </c>
-      <c r="N20" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+      <c r="N20"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="Q20"/>
+    </row>
+    <row r="21" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="B21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" t="s">
         <v>38</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21"/>
+      <c r="E21" t="s">
         <v>39</v>
       </c>
-      <c r="E21" t="s">
-        <v>75</v>
-      </c>
       <c r="F21" t="s">
-        <v>128</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="G21"/>
+      <c r="H21"/>
       <c r="I21" t="b">
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>36</v>
+        <v>53</v>
+      </c>
+      <c r="K21" t="s">
+        <v>57</v>
       </c>
       <c r="L21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M21" t="s">
-        <v>33</v>
-      </c>
-      <c r="N21" t="s">
-        <v>33</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="N21"/>
+      <c r="O21"/>
+      <c r="P21"/>
+      <c r="Q21"/>
     </row>
     <row r="22" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="B22" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D22"/>
       <c r="E22" t="s">
-        <v>136</v>
+        <v>39</v>
       </c>
       <c r="F22" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="G22"/>
       <c r="H22"/>
       <c r="I22" t="b">
         <v>1</v>
       </c>
-      <c r="J22"/>
+      <c r="J22" t="s">
+        <v>33</v>
+      </c>
       <c r="K22" t="s">
-        <v>130</v>
-      </c>
-      <c r="L22"/>
+        <v>56</v>
+      </c>
+      <c r="L22" t="s">
+        <v>34</v>
+      </c>
       <c r="M22" t="s">
-        <v>33</v>
+        <v>99</v>
       </c>
       <c r="N22"/>
-      <c r="O22" t="s">
-        <v>35</v>
-      </c>
+      <c r="O22"/>
       <c r="P22"/>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="Q22"/>
+    </row>
+    <row r="23" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
+        <v>38</v>
+      </c>
+      <c r="D23"/>
+      <c r="E23" t="s">
         <v>39</v>
       </c>
-      <c r="E23" t="s">
-        <v>136</v>
-      </c>
       <c r="F23" t="s">
-        <v>131</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="G23"/>
+      <c r="H23"/>
       <c r="I23" t="b">
         <v>1</v>
       </c>
+      <c r="J23" t="s">
+        <v>33</v>
+      </c>
       <c r="K23" t="s">
-        <v>73</v>
+        <v>56</v>
+      </c>
+      <c r="L23" t="s">
+        <v>99</v>
       </c>
       <c r="M23" t="s">
+        <v>32</v>
+      </c>
+      <c r="N23"/>
+      <c r="O23"/>
+      <c r="P23"/>
+      <c r="Q23"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" t="s">
+        <v>39</v>
+      </c>
+      <c r="F24" t="s">
+        <v>155</v>
+      </c>
+      <c r="I24" t="b">
+        <v>1</v>
+      </c>
+      <c r="J24" t="s">
+        <v>35</v>
+      </c>
+      <c r="K24" t="s">
+        <v>56</v>
+      </c>
+      <c r="L24" t="s">
+        <v>34</v>
+      </c>
+      <c r="M24" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>117</v>
+      </c>
+      <c r="B25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25"/>
+      <c r="E25" t="s">
+        <v>68</v>
+      </c>
+      <c r="F25" t="s">
+        <v>118</v>
+      </c>
+      <c r="G25"/>
+      <c r="H25"/>
+      <c r="I25" t="b">
+        <v>1</v>
+      </c>
+      <c r="J25" t="s">
         <v>33</v>
       </c>
-      <c r="O23" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J24" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="K24" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="L24" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="M24" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>84</v>
-      </c>
       <c r="K25"/>
-      <c r="L25" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="M25"/>
-      <c r="N25"/>
+      <c r="L25" t="s">
+        <v>34</v>
+      </c>
+      <c r="M25" t="s">
+        <v>99</v>
+      </c>
+      <c r="N25" t="s">
+        <v>32</v>
+      </c>
       <c r="O25"/>
       <c r="P25"/>
+      <c r="Q25"/>
     </row>
     <row r="26" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J26" s="8" t="s">
+      <c r="A26" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26"/>
+      <c r="E26" t="s">
+        <v>68</v>
+      </c>
+      <c r="F26" t="s">
+        <v>119</v>
+      </c>
+      <c r="G26"/>
+      <c r="H26"/>
+      <c r="I26" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" t="s">
+        <v>33</v>
+      </c>
+      <c r="K26"/>
+      <c r="L26" t="s">
+        <v>99</v>
+      </c>
+      <c r="M26" t="s">
+        <v>32</v>
+      </c>
+      <c r="N26" t="s">
+        <v>32</v>
+      </c>
+      <c r="O26"/>
+      <c r="P26"/>
+      <c r="Q26"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>117</v>
+      </c>
+      <c r="B27" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" t="s">
+        <v>38</v>
+      </c>
+      <c r="E27" t="s">
+        <v>68</v>
+      </c>
+      <c r="F27" t="s">
+        <v>120</v>
+      </c>
+      <c r="I27" t="b">
+        <v>1</v>
+      </c>
+      <c r="J27" t="s">
+        <v>35</v>
+      </c>
+      <c r="L27" t="s">
+        <v>34</v>
+      </c>
+      <c r="M27" t="s">
+        <v>32</v>
+      </c>
+      <c r="N27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>121</v>
+      </c>
+      <c r="B28" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28"/>
+      <c r="E28" t="s">
+        <v>122</v>
+      </c>
+      <c r="F28" t="s">
+        <v>121</v>
+      </c>
+      <c r="G28"/>
+      <c r="H28"/>
+      <c r="I28" t="b">
+        <v>1</v>
+      </c>
+      <c r="J28"/>
+      <c r="K28" t="s">
+        <v>123</v>
+      </c>
+      <c r="L28"/>
+      <c r="M28" t="s">
+        <v>32</v>
+      </c>
+      <c r="N28"/>
+      <c r="O28" t="s">
+        <v>34</v>
+      </c>
+      <c r="P28"/>
+      <c r="Q28"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" t="s">
+        <v>38</v>
+      </c>
+      <c r="E29" t="s">
+        <v>122</v>
+      </c>
+      <c r="F29" t="s">
+        <v>163</v>
+      </c>
+      <c r="I29" t="b">
+        <v>1</v>
+      </c>
+      <c r="K29" t="s">
+        <v>123</v>
+      </c>
+      <c r="M29" t="s">
+        <v>99</v>
+      </c>
+      <c r="O29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A30" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="K26" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="L26" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="M26" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="J27" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="L27" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="O28" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="F29" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="K29" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="M29" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="8" t="s">
-        <v>92</v>
-      </c>
       <c r="B30" s="8" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>16</v>
       </c>
+      <c r="D30" s="8"/>
       <c r="E30" s="8" t="s">
-        <v>68</v>
+        <v>23</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="K30" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="M30" s="8" t="s">
-        <v>35</v>
+        <v>75</v>
+      </c>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="L30" s="8" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="8" t="s">
-        <v>95</v>
+        <v>165</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>97</v>
+        <v>39</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>95</v>
+        <v>165</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>69</v>
+        <v>61</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="L31" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="M31" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="N31" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="32" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="8" t="s">
-        <v>107</v>
+        <v>51</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>107</v>
+        <v>51</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="K32" s="8" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="L32" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M32" s="8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="8" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>47</v>
+        <v>80</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>16</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="K33" s="8" t="s">
-        <v>34</v>
+        <v>63</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="L33" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="M33" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="8" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D34" s="8"/>
       <c r="E34" s="8" t="s">
-        <v>74</v>
+        <v>124</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="H34" s="8"/>
-      <c r="I34" s="8"/>
-      <c r="J34" s="8"/>
-      <c r="K34" s="8"/>
-      <c r="L34" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="M34" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="N34" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="O34" s="8"/>
-      <c r="P34" s="8"/>
-    </row>
-    <row r="35" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+      <c r="O34" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="8" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D35" s="8"/>
       <c r="E35" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="M35" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="M36" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G37" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="M37" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N37" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G38" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="K38" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="L38" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M38" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G39" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="K39" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L39" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M39" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L40" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M40" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="N40" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="G41" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J41" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="K41" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="L41" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M41" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J42" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="L42" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="M42" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E43" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F35" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="M35" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="8"/>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A36" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="C36" s="9" t="s">
+      <c r="F43" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="J43" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="K43" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>87</v>
+      </c>
+      <c r="B44" t="s">
+        <v>88</v>
+      </c>
+      <c r="C44" t="s">
         <v>15</v>
       </c>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="9"/>
-      <c r="J36" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="K36" s="9"/>
-      <c r="L36" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="M36" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="N36" s="9"/>
-      <c r="O36" s="9"/>
-      <c r="P36" s="9"/>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A37" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="B37" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C37" s="9" t="s">
+      <c r="E44" t="s">
+        <v>89</v>
+      </c>
+      <c r="F44" t="s">
+        <v>90</v>
+      </c>
+      <c r="P44" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>87</v>
+      </c>
+      <c r="B45" t="s">
+        <v>88</v>
+      </c>
+      <c r="C45" t="s">
         <v>15</v>
       </c>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="G37" s="9"/>
-      <c r="H37" s="9"/>
-      <c r="I37" s="9"/>
-      <c r="J37" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="K37" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="L37" s="9"/>
-      <c r="M37" s="9"/>
-      <c r="N37" s="9"/>
-      <c r="O37" s="9"/>
-      <c r="P37" s="9"/>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>98</v>
-      </c>
-      <c r="B38" t="s">
-        <v>99</v>
-      </c>
-      <c r="C38" t="s">
-        <v>15</v>
-      </c>
-      <c r="E38" t="s">
-        <v>100</v>
-      </c>
-      <c r="F38" t="s">
-        <v>101</v>
-      </c>
-      <c r="P38" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>98</v>
-      </c>
-      <c r="B39" t="s">
-        <v>99</v>
-      </c>
-      <c r="C39" t="s">
-        <v>15</v>
-      </c>
-      <c r="E39" t="s">
-        <v>100</v>
-      </c>
-      <c r="F39" t="s">
-        <v>103</v>
-      </c>
-      <c r="P39" t="s">
-        <v>104</v>
+      <c r="E45" t="s">
+        <v>89</v>
+      </c>
+      <c r="F45" t="s">
+        <v>92</v>
+      </c>
+      <c r="P45" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N23" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}"/>
+  <autoFilter ref="A1:N30" xr:uid="{99EF8F26-7547-4076-9880-E796E9F04B5A}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="3916dc5588df290b35e5c499b507bc33">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e3fae628afbc47c424dc6703fd07071" ns2:_="" ns3:_="">
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="90e7079a-7589-470d-892b-836f3f5ab9a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9ef6bf99-292f-445d-95df-6a8984d5eb85" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="348072715f26cde881c56d84fe7c6dcc">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="53f9bc5e977a2cc0a870214cffd63ac6" ns2:_="" ns3:_="">
     <xsd:import namespace="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
     <xsd:import namespace="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
     <xsd:element name="properties">
@@ -2373,7 +2698,7 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Tag immagine" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -2427,8 +2752,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo di contenuto"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titolo"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -2517,41 +2842,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="90e7079a-7589-470d-892b-836f3f5ab9a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9ef6bf99-292f-445d-95df-6a8984d5eb85" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D513A36A-455A-47E3-AF12-8A71C090EFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91788BB2-4A3F-4B3D-BB9A-4A497CBAE5D7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
-    <ds:schemaRef ds:uri="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2574,9 +2868,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91788BB2-4A3F-4B3D-BB9A-4A497CBAE5D7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2B120C4-3E0A-4AEB-AE39-18AAEAF48069}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
+    <ds:schemaRef ds:uri="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>